<commit_message>
Monica : revue du script global et intros/outros E1–E5 ; scripts E22.
Aligner les parties B sur sujet + présentation de l’expert, outro à retenir et projection vers la vidéo suivante.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/site/suivi_positionnements.xlsx
+++ b/site/suivi_positionnements.xlsx
@@ -799,10 +799,15 @@
           <t>T12 (E22, E23)</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr"/>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11 — Script revu/corrigé reçu (voix cellule partenariats UPS : point d’entrée, prospection, collaboration vs prestation, NDA, dimensionnement, négociation, six repères, chute public-privé). Déposé scripts_recus/E22.txt ; prompteur scripts_valides/E22.txt (coquilles seulement).</t>
+        </is>
+      </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08 — Demande un script déjà rédigé, avec peu de retouches. Proposition déposée (briefs/remi_wache_E22.txt + E22_proposition.json), ~747 mots / 5 min. Ancrage T12 monté (dispositifs, introductions, pitch, cohorte) ; frontière nette avec E23 (Eneli Vino). Tournage 11/09 09:00.</t>
+          <t>2026-09-08 — Demande un script déjà rédigé, avec peu de retouches. Proposition déposée (briefs/remi_wache_E22.txt + E22_proposition.json).
+2026-09-11 — Version Rémi arrêtée pour tournage (~1200 mots / ~8 min). Recouvrement E23 conservé (renvoi à la vidéo suivante).</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Aligner les scripts finaux des vidéos expert filmées le 24 septembre.
Les textes fournis (E3, E12, E13, E15, E17, E18) sont en reçu et validé ; les 15 V0 du 7–11 septembre restent la source filmée.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/site/suivi_positionnements.xlsx
+++ b/site/suivi_positionnements.xlsx
@@ -499,7 +499,8 @@
       <c r="E2" s="2" t="inlineStr">
         <is>
           <t>2026-09-10 — Proposition de script E17 (briefs/antoine_latreille_E17.txt). Ancrage T9 ; frontière E16. Oral : pacte d'associés, sans mention de la loi PACTE.
-2026-09-24 — Filmé E17 (10:30, IncubAlliance). V0 pas encore importé.</t>
+2026-09-24 — Filmé E17 (10:30, IncubAlliance).
+2026-09-25 — Script final = texte fourni par Antoine (scripts_recus/E17.txt, scripts_valides/E17.txt). Éléments de langage PI (FTO, NDA, etc.) exclus du script final.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr"/>
@@ -528,7 +529,8 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 — Filmé E13, E15, E18 (09:00, IncubAlliance). V0 pas encore importé.</t>
+          <t>2026-09-24 — Filmé E13, E15, E18 (09:00, IncubAlliance). V0 pas encore importé.
+2026-09-25 — Scripts finaux = textes fournis par Arielle (recus + valides E13, E15, E18), déposés tels quels.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr"/>
@@ -685,7 +687,8 @@
       <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Point à la rentrée pour clarifier le lien script / sujets expert et cadrer l'intervention. Préfère parler sans script pré-écrit.
-2026-09-24 — Filmé E3 (14:30, IncubAlliance). V0 pas encore importé.</t>
+2026-09-24 — Filmé E3 (14:30, IncubAlliance). V0 pas encore importé.
+2026-09-25 — Script final = texte fourni par Grégoire (scripts_recus/E3.txt, scripts_valides/E3.txt). Texte tel quel, sans réécriture. Techno-push / market-pull : contraste pour renforcer le market-pull, pas une leçon d'origines (E1). Frontière E2 à recadrer ensuite côté Joël (pas encore tourné).</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">

</xml_diff>